<commit_message>
fix some testcase for app and add docs
</commit_message>
<xml_diff>
--- a/KICHBAN_TEST_KHACH_HANG_HealthyAI.xlsx
+++ b/KICHBAN_TEST_KHACH_HANG_HealthyAI.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\HealthyAIApp\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\KMA\LapTrinhAndroidNangCao\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{749D14F6-FA7D-4B9D-93C7-12F9EE2D9BB1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95412B3B-F904-4B32-AEA4-58D17352D468}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hướng dẫn" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1213" uniqueCount="638">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1229" uniqueCount="644">
   <si>
     <t>STT</t>
   </si>
@@ -1960,6 +1960,24 @@
   </si>
   <si>
     <t>Hết tài liệu. Khi test xong, gửi lại mục 8 (bảng theo dõi) + các vấn đề ở mục 7 cho nhóm phát triển.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">  </t>
+  </si>
+  <si>
+    <t>Thẻ rest về 0/45</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ko hiển thị thẻ </t>
+  </si>
+  <si>
+    <t>nhảy sang tab Thói quen mà không mở hộp thoại nào</t>
+  </si>
+  <si>
+    <t>máy thật có cảm biến mà không thấy thẻ</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ko có thẻ "Bật nhắc nhở hàng ngày" </t>
   </si>
 </sst>
 </file>
@@ -2129,9 +2147,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 - 2022 Theme">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -2169,7 +2187,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -2275,7 +2293,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -2417,7 +2435,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -2425,408 +2443,411 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:A88"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:I88"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="128" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>422</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6" t="s">
         <v>423</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="7" t="s">
         <v>424</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>425</v>
       </c>
-    </row>
-    <row r="7" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="I6" t="s">
+        <v>638</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>426</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>427</v>
       </c>
     </row>
-    <row r="9" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>428</v>
       </c>
     </row>
-    <row r="10" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>429</v>
       </c>
     </row>
-    <row r="11" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>430</v>
       </c>
     </row>
-    <row r="13" spans="1:1" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>431</v>
       </c>
     </row>
-    <row r="15" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
         <v>432</v>
       </c>
     </row>
-    <row r="16" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
         <v>433</v>
       </c>
     </row>
-    <row r="17" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>434</v>
       </c>
     </row>
-    <row r="18" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>435</v>
       </c>
     </row>
-    <row r="19" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>436</v>
       </c>
     </row>
-    <row r="20" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="7" t="s">
         <v>437</v>
       </c>
     </row>
-    <row r="21" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>438</v>
       </c>
     </row>
-    <row r="22" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>439</v>
       </c>
     </row>
-    <row r="23" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>440</v>
       </c>
     </row>
-    <row r="24" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>441</v>
       </c>
     </row>
-    <row r="25" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="7" t="s">
         <v>442</v>
       </c>
     </row>
-    <row r="26" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
         <v>443</v>
       </c>
     </row>
-    <row r="27" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
         <v>444</v>
       </c>
     </row>
-    <row r="29" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
         <v>445</v>
       </c>
     </row>
-    <row r="30" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="7" t="s">
         <v>446</v>
       </c>
     </row>
-    <row r="31" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
         <v>447</v>
       </c>
     </row>
-    <row r="32" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
         <v>448</v>
       </c>
     </row>
-    <row r="33" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
         <v>449</v>
       </c>
     </row>
-    <row r="34" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
         <v>450</v>
       </c>
     </row>
-    <row r="35" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
         <v>451</v>
       </c>
     </row>
-    <row r="36" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="7" t="s">
         <v>452</v>
       </c>
     </row>
-    <row r="37" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="6" t="s">
         <v>453</v>
       </c>
     </row>
-    <row r="38" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
         <v>454</v>
       </c>
     </row>
-    <row r="39" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="7" t="s">
         <v>455</v>
       </c>
     </row>
-    <row r="40" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
         <v>456</v>
       </c>
     </row>
-    <row r="41" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
         <v>457</v>
       </c>
     </row>
-    <row r="42" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="6" t="s">
         <v>458</v>
       </c>
     </row>
-    <row r="43" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
         <v>459</v>
       </c>
     </row>
-    <row r="44" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="7" t="s">
         <v>460</v>
       </c>
     </row>
-    <row r="45" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="6" t="s">
         <v>461</v>
       </c>
     </row>
-    <row r="46" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
         <v>462</v>
       </c>
     </row>
-    <row r="47" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
         <v>463</v>
       </c>
     </row>
-    <row r="48" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="8" t="s">
         <v>464</v>
       </c>
     </row>
-    <row r="50" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="7" t="s">
         <v>465</v>
       </c>
     </row>
-    <row r="51" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="6" t="s">
         <v>466</v>
       </c>
     </row>
-    <row r="52" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
         <v>467</v>
       </c>
     </row>
-    <row r="53" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
         <v>468</v>
       </c>
     </row>
-    <row r="54" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
         <v>469</v>
       </c>
     </row>
-    <row r="55" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="6" t="s">
         <v>470</v>
       </c>
     </row>
-    <row r="56" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="6" t="s">
         <v>471</v>
       </c>
     </row>
-    <row r="57" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="6" t="s">
         <v>472</v>
       </c>
     </row>
-    <row r="58" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="6" t="s">
         <v>473</v>
       </c>
     </row>
-    <row r="59" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="6" t="s">
         <v>474</v>
       </c>
     </row>
-    <row r="60" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="6" t="s">
         <v>475</v>
       </c>
     </row>
-    <row r="61" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="6" t="s">
         <v>476</v>
       </c>
     </row>
-    <row r="62" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="6" t="s">
         <v>477</v>
       </c>
     </row>
-    <row r="63" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="6" t="s">
         <v>478</v>
       </c>
     </row>
-    <row r="64" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="6" t="s">
         <v>479</v>
       </c>
     </row>
-    <row r="65" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="6" t="s">
         <v>480</v>
       </c>
     </row>
-    <row r="66" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="6" t="s">
         <v>481</v>
       </c>
     </row>
-    <row r="68" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="7" t="s">
         <v>482</v>
       </c>
     </row>
-    <row r="69" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="6" t="s">
         <v>483</v>
       </c>
     </row>
-    <row r="70" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="6" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="71" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="6" t="s">
         <v>484</v>
       </c>
     </row>
-    <row r="72" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="6" t="s">
         <v>485</v>
       </c>
     </row>
-    <row r="73" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="6" t="s">
         <v>486</v>
       </c>
     </row>
-    <row r="74" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="6" t="s">
         <v>487</v>
       </c>
     </row>
-    <row r="75" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="6" t="s">
         <v>488</v>
       </c>
     </row>
-    <row r="76" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="6" t="s">
         <v>489</v>
       </c>
     </row>
-    <row r="77" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="6" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="78" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="6" t="s">
         <v>490</v>
       </c>
     </row>
-    <row r="79" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="6" t="s">
         <v>491</v>
       </c>
     </row>
-    <row r="80" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="6" t="s">
         <v>492</v>
       </c>
     </row>
-    <row r="81" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="6" t="s">
         <v>493</v>
       </c>
     </row>
-    <row r="82" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="6" t="s">
         <v>494</v>
       </c>
     </row>
-    <row r="83" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="8" t="s">
         <v>495</v>
       </c>
     </row>
-    <row r="85" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="7" t="s">
         <v>496</v>
       </c>
     </row>
-    <row r="86" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A86" s="6" t="s">
         <v>497</v>
       </c>
     </row>
-    <row r="87" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="6" t="s">
         <v>498</v>
       </c>
     </row>
-    <row r="88" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="6" t="s">
         <v>499</v>
       </c>
@@ -2839,7 +2860,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:M81"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5" customWidth="1"/>
     <col min="2" max="2" width="8" customWidth="1"/>
@@ -2855,7 +2876,7 @@
     <col min="13" max="13" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -2896,7 +2917,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="84.45" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" ht="84.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="4">
         <v>1</v>
       </c>
@@ -2924,10 +2945,10 @@
       <c r="I2" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="J2" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="K2" s="4"/>
+      <c r="J2" s="2"/>
+      <c r="K2" s="4" t="s">
+        <v>505</v>
+      </c>
       <c r="L2" s="2" t="s">
         <v>21</v>
       </c>
@@ -2935,7 +2956,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="4">
         <v>2</v>
       </c>
@@ -2967,7 +2988,7 @@
         <v>21</v>
       </c>
       <c r="K3" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L3" s="2" t="s">
         <v>21</v>
@@ -2976,7 +2997,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="4" spans="1:13" ht="70.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:13" ht="70.900000000000006" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="4">
         <v>3</v>
       </c>
@@ -3008,7 +3029,7 @@
         <v>21</v>
       </c>
       <c r="K4" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L4" s="2" t="s">
         <v>21</v>
@@ -3017,7 +3038,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="4">
         <v>4</v>
       </c>
@@ -3049,7 +3070,7 @@
         <v>39</v>
       </c>
       <c r="K5" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L5" s="2" t="s">
         <v>21</v>
@@ -3058,7 +3079,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="4">
         <v>5</v>
       </c>
@@ -3090,7 +3111,7 @@
         <v>21</v>
       </c>
       <c r="K6" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L6" s="2" t="s">
         <v>21</v>
@@ -3099,7 +3120,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="97.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" ht="97.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="4">
         <v>6</v>
       </c>
@@ -3131,7 +3152,7 @@
         <v>21</v>
       </c>
       <c r="K7" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L7" s="2" t="s">
         <v>21</v>
@@ -3140,7 +3161,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="70.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" ht="70.900000000000006" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4">
         <v>7</v>
       </c>
@@ -3172,7 +3193,7 @@
         <v>21</v>
       </c>
       <c r="K8" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L8" s="2" t="s">
         <v>21</v>
@@ -3181,7 +3202,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="84.45" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" ht="84.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="4">
         <v>8</v>
       </c>
@@ -3213,7 +3234,7 @@
         <v>21</v>
       </c>
       <c r="K9" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L9" s="2" t="s">
         <v>21</v>
@@ -3222,7 +3243,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="4">
         <v>9</v>
       </c>
@@ -3254,7 +3275,7 @@
         <v>21</v>
       </c>
       <c r="K10" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L10" s="2" t="s">
         <v>21</v>
@@ -3263,7 +3284,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="4">
         <v>10</v>
       </c>
@@ -3295,7 +3316,7 @@
         <v>21</v>
       </c>
       <c r="K11" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L11" s="2" t="s">
         <v>21</v>
@@ -3304,7 +3325,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="4">
         <v>11</v>
       </c>
@@ -3336,7 +3357,7 @@
         <v>21</v>
       </c>
       <c r="K12" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L12" s="2" t="s">
         <v>21</v>
@@ -3345,7 +3366,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="4">
         <v>12</v>
       </c>
@@ -3377,7 +3398,7 @@
         <v>21</v>
       </c>
       <c r="K13" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L13" s="2" t="s">
         <v>21</v>
@@ -3386,7 +3407,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="4">
         <v>13</v>
       </c>
@@ -3418,16 +3439,16 @@
         <v>21</v>
       </c>
       <c r="K14" s="4" t="s">
-        <v>21</v>
+        <v>506</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>21</v>
+        <v>639</v>
       </c>
       <c r="M14" s="4" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="4">
         <v>14</v>
       </c>
@@ -3459,7 +3480,7 @@
         <v>21</v>
       </c>
       <c r="K15" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L15" s="2" t="s">
         <v>21</v>
@@ -3468,7 +3489,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="70.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:13" ht="70.900000000000006" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="4">
         <v>15</v>
       </c>
@@ -3500,7 +3521,7 @@
         <v>21</v>
       </c>
       <c r="K16" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L16" s="2" t="s">
         <v>21</v>
@@ -3509,7 +3530,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="17" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="4">
         <v>16</v>
       </c>
@@ -3541,7 +3562,7 @@
         <v>21</v>
       </c>
       <c r="K17" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L17" s="2" t="s">
         <v>21</v>
@@ -3550,7 +3571,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="18" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="4">
         <v>17</v>
       </c>
@@ -3582,7 +3603,7 @@
         <v>21</v>
       </c>
       <c r="K18" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L18" s="2" t="s">
         <v>21</v>
@@ -3591,7 +3612,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="19" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="4">
         <v>18</v>
       </c>
@@ -3623,7 +3644,7 @@
         <v>21</v>
       </c>
       <c r="K19" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L19" s="2" t="s">
         <v>21</v>
@@ -3632,7 +3653,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="20" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="4">
         <v>19</v>
       </c>
@@ -3664,7 +3685,7 @@
         <v>21</v>
       </c>
       <c r="K20" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L20" s="2" t="s">
         <v>21</v>
@@ -3673,7 +3694,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="4">
         <v>20</v>
       </c>
@@ -3705,7 +3726,7 @@
         <v>21</v>
       </c>
       <c r="K21" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L21" s="2" t="s">
         <v>21</v>
@@ -3714,7 +3735,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="22" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="4">
         <v>21</v>
       </c>
@@ -3746,7 +3767,7 @@
         <v>21</v>
       </c>
       <c r="K22" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L22" s="2" t="s">
         <v>21</v>
@@ -3755,7 +3776,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="23" spans="1:13" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:13" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="4">
         <v>22</v>
       </c>
@@ -3787,7 +3808,7 @@
         <v>21</v>
       </c>
       <c r="K23" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L23" s="2" t="s">
         <v>21</v>
@@ -3796,7 +3817,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="24" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="4">
         <v>23</v>
       </c>
@@ -3828,7 +3849,7 @@
         <v>21</v>
       </c>
       <c r="K24" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L24" s="2" t="s">
         <v>21</v>
@@ -3837,7 +3858,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="25" spans="1:13" ht="70.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:13" ht="70.900000000000006" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="4">
         <v>24</v>
       </c>
@@ -3869,7 +3890,7 @@
         <v>21</v>
       </c>
       <c r="K25" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L25" s="2" t="s">
         <v>21</v>
@@ -3878,7 +3899,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="26" spans="1:13" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:13" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="4">
         <v>25</v>
       </c>
@@ -3910,7 +3931,7 @@
         <v>21</v>
       </c>
       <c r="K26" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L26" s="2" t="s">
         <v>21</v>
@@ -3919,7 +3940,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="27" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="4">
         <v>26</v>
       </c>
@@ -3951,7 +3972,7 @@
         <v>21</v>
       </c>
       <c r="K27" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L27" s="2" t="s">
         <v>21</v>
@@ -3960,7 +3981,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="28" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="4">
         <v>27</v>
       </c>
@@ -3992,7 +4013,7 @@
         <v>21</v>
       </c>
       <c r="K28" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L28" s="2" t="s">
         <v>21</v>
@@ -4001,7 +4022,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="29" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="4">
         <v>28</v>
       </c>
@@ -4033,7 +4054,7 @@
         <v>21</v>
       </c>
       <c r="K29" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L29" s="2" t="s">
         <v>21</v>
@@ -4042,7 +4063,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="30" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="4">
         <v>29</v>
       </c>
@@ -4074,7 +4095,7 @@
         <v>21</v>
       </c>
       <c r="K30" s="4" t="s">
-        <v>21</v>
+        <v>507</v>
       </c>
       <c r="L30" s="2" t="s">
         <v>21</v>
@@ -4083,7 +4104,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="31" spans="1:13" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:13" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="4">
         <v>30</v>
       </c>
@@ -4115,7 +4136,7 @@
         <v>21</v>
       </c>
       <c r="K31" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L31" s="2" t="s">
         <v>21</v>
@@ -4124,7 +4145,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="32" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="4">
         <v>31</v>
       </c>
@@ -4156,7 +4177,7 @@
         <v>21</v>
       </c>
       <c r="K32" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L32" s="2" t="s">
         <v>21</v>
@@ -4165,7 +4186,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="33" spans="1:13" ht="151.35" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:13" ht="151.35" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="4">
         <v>32</v>
       </c>
@@ -4197,7 +4218,7 @@
         <v>179</v>
       </c>
       <c r="K33" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L33" s="2" t="s">
         <v>21</v>
@@ -4206,7 +4227,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="34" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="4">
         <v>33</v>
       </c>
@@ -4238,7 +4259,7 @@
         <v>21</v>
       </c>
       <c r="K34" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L34" s="2" t="s">
         <v>21</v>
@@ -4247,7 +4268,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="35" spans="1:13" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:13" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="4">
         <v>34</v>
       </c>
@@ -4279,7 +4300,7 @@
         <v>21</v>
       </c>
       <c r="K35" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L35" s="2" t="s">
         <v>21</v>
@@ -4288,7 +4309,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="36" spans="1:13" ht="70.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:13" ht="70.900000000000006" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="4">
         <v>35</v>
       </c>
@@ -4320,7 +4341,7 @@
         <v>192</v>
       </c>
       <c r="K36" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L36" s="2" t="s">
         <v>21</v>
@@ -4329,7 +4350,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="37" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="4">
         <v>36</v>
       </c>
@@ -4361,16 +4382,16 @@
         <v>21</v>
       </c>
       <c r="K37" s="4" t="s">
-        <v>21</v>
+        <v>506</v>
       </c>
       <c r="L37" s="2" t="s">
-        <v>21</v>
+        <v>643</v>
       </c>
       <c r="M37" s="4" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="38" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="4">
         <v>37</v>
       </c>
@@ -4402,16 +4423,16 @@
         <v>21</v>
       </c>
       <c r="K38" s="4" t="s">
-        <v>21</v>
+        <v>506</v>
       </c>
       <c r="L38" s="2" t="s">
-        <v>21</v>
+        <v>643</v>
       </c>
       <c r="M38" s="4" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="39" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="4">
         <v>38</v>
       </c>
@@ -4443,16 +4464,16 @@
         <v>21</v>
       </c>
       <c r="K39" s="4" t="s">
-        <v>21</v>
+        <v>506</v>
       </c>
       <c r="L39" s="2" t="s">
-        <v>21</v>
+        <v>640</v>
       </c>
       <c r="M39" s="4" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="40" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="4">
         <v>39</v>
       </c>
@@ -4484,16 +4505,14 @@
         <v>21</v>
       </c>
       <c r="K40" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="L40" s="2" t="s">
-        <v>21</v>
-      </c>
+        <v>505</v>
+      </c>
+      <c r="L40" s="2"/>
       <c r="M40" s="4" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="41" spans="1:13" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:13" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="4">
         <v>40</v>
       </c>
@@ -4525,7 +4544,7 @@
         <v>21</v>
       </c>
       <c r="K41" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L41" s="2" t="s">
         <v>21</v>
@@ -4534,7 +4553,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="42" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="4">
         <v>41</v>
       </c>
@@ -4566,7 +4585,7 @@
         <v>21</v>
       </c>
       <c r="K42" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L42" s="2" t="s">
         <v>21</v>
@@ -4575,7 +4594,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="43" spans="1:13" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:13" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="4">
         <v>42</v>
       </c>
@@ -4607,7 +4626,7 @@
         <v>21</v>
       </c>
       <c r="K43" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L43" s="2" t="s">
         <v>21</v>
@@ -4616,7 +4635,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="44" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="4">
         <v>43</v>
       </c>
@@ -4648,7 +4667,7 @@
         <v>21</v>
       </c>
       <c r="K44" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L44" s="2" t="s">
         <v>21</v>
@@ -4657,7 +4676,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="45" spans="1:13" ht="97.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:13" ht="97.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="4">
         <v>44</v>
       </c>
@@ -4689,7 +4708,7 @@
         <v>237</v>
       </c>
       <c r="K45" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L45" s="2" t="s">
         <v>21</v>
@@ -4698,7 +4717,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="46" spans="1:13" ht="84.45" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:13" ht="84.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="4">
         <v>45</v>
       </c>
@@ -4730,16 +4749,16 @@
         <v>243</v>
       </c>
       <c r="K46" s="4" t="s">
-        <v>21</v>
+        <v>506</v>
       </c>
       <c r="L46" s="2" t="s">
-        <v>21</v>
+        <v>641</v>
       </c>
       <c r="M46" s="4" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="47" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="4">
         <v>46</v>
       </c>
@@ -4771,7 +4790,7 @@
         <v>21</v>
       </c>
       <c r="K47" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L47" s="2" t="s">
         <v>21</v>
@@ -4780,7 +4799,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="48" spans="1:13" ht="97.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:13" ht="97.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="4">
         <v>47</v>
       </c>
@@ -4812,7 +4831,7 @@
         <v>21</v>
       </c>
       <c r="K48" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L48" s="2" t="s">
         <v>21</v>
@@ -4821,7 +4840,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="49" spans="1:13" ht="97.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:13" ht="97.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="4">
         <v>48</v>
       </c>
@@ -4853,7 +4872,7 @@
         <v>21</v>
       </c>
       <c r="K49" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L49" s="2" t="s">
         <v>21</v>
@@ -4862,7 +4881,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="50" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="4">
         <v>49</v>
       </c>
@@ -4894,7 +4913,7 @@
         <v>21</v>
       </c>
       <c r="K50" s="4" t="s">
-        <v>21</v>
+        <v>507</v>
       </c>
       <c r="L50" s="2" t="s">
         <v>21</v>
@@ -4903,7 +4922,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="51" spans="1:13" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:13" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="4">
         <v>50</v>
       </c>
@@ -4935,7 +4954,7 @@
         <v>21</v>
       </c>
       <c r="K51" s="4" t="s">
-        <v>21</v>
+        <v>507</v>
       </c>
       <c r="L51" s="2" t="s">
         <v>21</v>
@@ -4944,7 +4963,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="52" spans="1:13" ht="124.65" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:13" ht="124.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="4">
         <v>51</v>
       </c>
@@ -4976,7 +4995,7 @@
         <v>274</v>
       </c>
       <c r="K52" s="4" t="s">
-        <v>21</v>
+        <v>507</v>
       </c>
       <c r="L52" s="2" t="s">
         <v>21</v>
@@ -4985,7 +5004,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="53" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="4">
         <v>52</v>
       </c>
@@ -5017,7 +5036,7 @@
         <v>21</v>
       </c>
       <c r="K53" s="4" t="s">
-        <v>21</v>
+        <v>507</v>
       </c>
       <c r="L53" s="2" t="s">
         <v>21</v>
@@ -5026,7 +5045,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="54" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="4">
         <v>53</v>
       </c>
@@ -5058,7 +5077,7 @@
         <v>21</v>
       </c>
       <c r="K54" s="4" t="s">
-        <v>21</v>
+        <v>507</v>
       </c>
       <c r="L54" s="2" t="s">
         <v>21</v>
@@ -5067,7 +5086,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="55" spans="1:13" ht="70.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:13" ht="70.900000000000006" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="4">
         <v>54</v>
       </c>
@@ -5099,7 +5118,7 @@
         <v>21</v>
       </c>
       <c r="K55" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L55" s="2" t="s">
         <v>21</v>
@@ -5108,7 +5127,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="56" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="4">
         <v>55</v>
       </c>
@@ -5140,7 +5159,7 @@
         <v>21</v>
       </c>
       <c r="K56" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L56" s="2" t="s">
         <v>21</v>
@@ -5149,7 +5168,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="57" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="4">
         <v>56</v>
       </c>
@@ -5181,7 +5200,7 @@
         <v>21</v>
       </c>
       <c r="K57" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L57" s="2" t="s">
         <v>21</v>
@@ -5190,7 +5209,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="58" spans="1:13" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:13" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="4">
         <v>57</v>
       </c>
@@ -5222,7 +5241,7 @@
         <v>21</v>
       </c>
       <c r="K58" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L58" s="2" t="s">
         <v>21</v>
@@ -5231,7 +5250,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="59" spans="1:13" ht="84.45" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:13" ht="84.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="4">
         <v>58</v>
       </c>
@@ -5263,7 +5282,7 @@
         <v>311</v>
       </c>
       <c r="K59" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L59" s="2" t="s">
         <v>21</v>
@@ -5272,7 +5291,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="60" spans="1:13" ht="84.45" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:13" ht="84.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="4">
         <v>59</v>
       </c>
@@ -5304,7 +5323,7 @@
         <v>317</v>
       </c>
       <c r="K60" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L60" s="2" t="s">
         <v>21</v>
@@ -5313,7 +5332,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="61" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="4">
         <v>60</v>
       </c>
@@ -5345,7 +5364,7 @@
         <v>21</v>
       </c>
       <c r="K61" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L61" s="2" t="s">
         <v>21</v>
@@ -5354,7 +5373,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="62" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="4">
         <v>61</v>
       </c>
@@ -5386,7 +5405,7 @@
         <v>21</v>
       </c>
       <c r="K62" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L62" s="2" t="s">
         <v>21</v>
@@ -5395,7 +5414,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="63" spans="1:13" ht="70.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:13" ht="70.900000000000006" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="4">
         <v>62</v>
       </c>
@@ -5427,7 +5446,7 @@
         <v>21</v>
       </c>
       <c r="K63" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L63" s="2" t="s">
         <v>21</v>
@@ -5436,7 +5455,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="64" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="4">
         <v>63</v>
       </c>
@@ -5468,7 +5487,7 @@
         <v>21</v>
       </c>
       <c r="K64" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L64" s="2" t="s">
         <v>21</v>
@@ -5477,7 +5496,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="65" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="4">
         <v>64</v>
       </c>
@@ -5509,7 +5528,7 @@
         <v>21</v>
       </c>
       <c r="K65" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L65" s="2" t="s">
         <v>21</v>
@@ -5518,7 +5537,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="66" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="4">
         <v>65</v>
       </c>
@@ -5550,7 +5569,7 @@
         <v>21</v>
       </c>
       <c r="K66" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L66" s="2" t="s">
         <v>21</v>
@@ -5559,7 +5578,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="67" spans="1:13" ht="84.45" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:13" ht="84.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="4">
         <v>66</v>
       </c>
@@ -5591,7 +5610,7 @@
         <v>352</v>
       </c>
       <c r="K67" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L67" s="2" t="s">
         <v>21</v>
@@ -5600,7 +5619,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="68" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="4">
         <v>67</v>
       </c>
@@ -5632,7 +5651,7 @@
         <v>21</v>
       </c>
       <c r="K68" s="4" t="s">
-        <v>21</v>
+        <v>507</v>
       </c>
       <c r="L68" s="2" t="s">
         <v>21</v>
@@ -5641,7 +5660,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="69" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="4">
         <v>68</v>
       </c>
@@ -5673,7 +5692,7 @@
         <v>21</v>
       </c>
       <c r="K69" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L69" s="2" t="s">
         <v>21</v>
@@ -5682,7 +5701,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="70" spans="1:13" ht="124.65" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:13" ht="124.7" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="4">
         <v>69</v>
       </c>
@@ -5714,7 +5733,7 @@
         <v>364</v>
       </c>
       <c r="K70" s="4" t="s">
-        <v>21</v>
+        <v>508</v>
       </c>
       <c r="L70" s="2" t="s">
         <v>21</v>
@@ -5723,7 +5742,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="71" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="4">
         <v>70</v>
       </c>
@@ -5755,7 +5774,7 @@
         <v>21</v>
       </c>
       <c r="K71" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L71" s="2" t="s">
         <v>21</v>
@@ -5764,7 +5783,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="72" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="4">
         <v>71</v>
       </c>
@@ -5796,7 +5815,7 @@
         <v>21</v>
       </c>
       <c r="K72" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L72" s="2" t="s">
         <v>21</v>
@@ -5805,7 +5824,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="73" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="4">
         <v>72</v>
       </c>
@@ -5837,7 +5856,7 @@
         <v>21</v>
       </c>
       <c r="K73" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L73" s="2" t="s">
         <v>21</v>
@@ -5846,7 +5865,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="74" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:13" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="4">
         <v>73</v>
       </c>
@@ -5878,7 +5897,7 @@
         <v>21</v>
       </c>
       <c r="K74" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L74" s="2" t="s">
         <v>21</v>
@@ -5887,7 +5906,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="75" spans="1:13" ht="84.45" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:13" ht="84.4" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="4">
         <v>74</v>
       </c>
@@ -5919,7 +5938,7 @@
         <v>21</v>
       </c>
       <c r="K75" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L75" s="2" t="s">
         <v>21</v>
@@ -5928,7 +5947,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="76" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="4">
         <v>75</v>
       </c>
@@ -5960,7 +5979,7 @@
         <v>21</v>
       </c>
       <c r="K76" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L76" s="2" t="s">
         <v>21</v>
@@ -5969,7 +5988,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="77" spans="1:13" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:13" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="4">
         <v>76</v>
       </c>
@@ -6001,7 +6020,7 @@
         <v>21</v>
       </c>
       <c r="K77" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L77" s="2" t="s">
         <v>21</v>
@@ -6010,7 +6029,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="78" spans="1:13" ht="97.8" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:13" ht="97.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A78" s="4">
         <v>77</v>
       </c>
@@ -6042,16 +6061,16 @@
         <v>21</v>
       </c>
       <c r="K78" s="4" t="s">
-        <v>21</v>
+        <v>506</v>
       </c>
       <c r="L78" s="2" t="s">
-        <v>21</v>
+        <v>642</v>
       </c>
       <c r="M78" s="4" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="79" spans="1:13" ht="57.6" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:13" ht="57.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="4">
         <v>78</v>
       </c>
@@ -6083,7 +6102,7 @@
         <v>21</v>
       </c>
       <c r="K79" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L79" s="2" t="s">
         <v>21</v>
@@ -6092,7 +6111,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="80" spans="1:13" ht="178.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:13" ht="178.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="4">
         <v>79</v>
       </c>
@@ -6124,7 +6143,7 @@
         <v>416</v>
       </c>
       <c r="K80" s="4" t="s">
-        <v>21</v>
+        <v>505</v>
       </c>
       <c r="L80" s="2" t="s">
         <v>21</v>
@@ -6133,7 +6152,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="81" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:13" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="4">
         <v>80</v>
       </c>
@@ -6165,7 +6184,7 @@
         <v>21</v>
       </c>
       <c r="K81" s="4" t="s">
-        <v>21</v>
+        <v>507</v>
       </c>
       <c r="L81" s="2" t="s">
         <v>21</v>
@@ -6204,28 +6223,28 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:D31"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34" customWidth="1"/>
     <col min="2" max="4" width="12" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>500</v>
       </c>
     </row>
-    <row r="2" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:4" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="6" t="s">
         <v>501</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="7" t="s">
         <v>502</v>
       </c>
     </row>
-    <row r="5" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:4" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>503</v>
       </c>
@@ -6233,52 +6252,52 @@
         <v>504</v>
       </c>
     </row>
-    <row r="6" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="2" t="s">
         <v>505</v>
       </c>
       <c r="B6" s="4">
         <f>COUNTIF('Kịch bản test'!$K$2:$K$81,"Đạt")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+        <v>65</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2" t="s">
         <v>506</v>
       </c>
       <c r="B7" s="4">
         <f>COUNTIF('Kịch bản test'!$K$2:$K$81,"Không đạt")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="8" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="2" t="s">
         <v>507</v>
       </c>
       <c r="B8" s="4">
         <f>COUNTIF('Kịch bản test'!$K$2:$K$81,"Chưa test được")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="9" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="9" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="2" t="s">
         <v>508</v>
       </c>
       <c r="B9" s="4">
         <f>COUNTIF('Kịch bản test'!$K$2:$K$81,"Không áp dụng")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="10" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="2" t="s">
         <v>509</v>
       </c>
       <c r="B10" s="4">
         <f>COUNTA('Kịch bản test'!$B$2:$B$81)-SUM(B6:B9)</f>
-        <v>80</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" ht="18" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="3" t="s">
         <v>510</v>
       </c>
@@ -6287,12 +6306,12 @@
         <v>80</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" s="7" t="s">
         <v>511</v>
       </c>
     </row>
-    <row r="14" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:4" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
         <v>3</v>
       </c>
@@ -6306,7 +6325,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" s="2" t="s">
         <v>15</v>
       </c>
@@ -6320,10 +6339,10 @@
       </c>
       <c r="D15" s="4">
         <f>COUNTIFS('Kịch bản test'!$D$2:$D$81,"Bắt buộc",'Kịch bản test'!$K$2:$K$81,"")</f>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="2" t="s">
         <v>29</v>
       </c>
@@ -6333,14 +6352,14 @@
       </c>
       <c r="C16" s="4">
         <f>COUNTIFS('Kịch bản test'!$D$2:$D$81,"Quan trọng",'Kịch bản test'!$K$2:$K$81,"Không đạt")</f>
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="D16" s="4">
         <f>COUNTIFS('Kịch bản test'!$D$2:$D$81,"Quan trọng",'Kịch bản test'!$K$2:$K$81,"")</f>
-        <v>50</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" s="2" t="s">
         <v>23</v>
       </c>
@@ -6354,15 +6373,15 @@
       </c>
       <c r="D17" s="4">
         <f>COUNTIFS('Kịch bản test'!$D$2:$D$81,"Tùy chọn",'Kịch bản test'!$K$2:$K$81,"")</f>
-        <v>20</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
         <v>514</v>
       </c>
     </row>
-    <row r="20" spans="1:4" ht="19.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:4" ht="19.899999999999999" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>2</v>
       </c>
@@ -6376,7 +6395,7 @@
         <v>513</v>
       </c>
     </row>
-    <row r="21" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="2" t="s">
         <v>14</v>
       </c>
@@ -6390,10 +6409,10 @@
       </c>
       <c r="D21" s="4">
         <f>COUNTIFS('Kịch bản test'!$C$2:$C$81,"Hành trình A*",'Kịch bản test'!$K$2:$K$81,"")</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="22" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="22" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="2" t="s">
         <v>61</v>
       </c>
@@ -6403,14 +6422,14 @@
       </c>
       <c r="C22" s="4">
         <f>COUNTIFS('Kịch bản test'!$C$2:$C$81,"Hành trình B*",'Kịch bản test'!$K$2:$K$81,"Không đạt")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D22" s="4">
         <f>COUNTIFS('Kịch bản test'!$C$2:$C$81,"Hành trình B*",'Kịch bản test'!$K$2:$K$81,"")</f>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="23" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="23" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="2" t="s">
         <v>111</v>
       </c>
@@ -6424,10 +6443,10 @@
       </c>
       <c r="D23" s="4">
         <f>COUNTIFS('Kịch bản test'!$C$2:$C$81,"Hành trình C*",'Kịch bản test'!$K$2:$K$81,"")</f>
-        <v>9</v>
-      </c>
-    </row>
-    <row r="24" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="2" t="s">
         <v>155</v>
       </c>
@@ -6441,10 +6460,10 @@
       </c>
       <c r="D24" s="4">
         <f>COUNTIFS('Kịch bản test'!$C$2:$C$81,"Hành trình D*",'Kịch bản test'!$K$2:$K$81,"")</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="25" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="25" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="2" t="s">
         <v>194</v>
       </c>
@@ -6454,14 +6473,14 @@
       </c>
       <c r="C25" s="4">
         <f>COUNTIFS('Kịch bản test'!$C$2:$C$81,"Hành trình E*",'Kịch bản test'!$K$2:$K$81,"Không đạt")</f>
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="D25" s="4">
         <f>COUNTIFS('Kịch bản test'!$C$2:$C$81,"Hành trình E*",'Kịch bản test'!$K$2:$K$81,"")</f>
-        <v>6</v>
-      </c>
-    </row>
-    <row r="26" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="26" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="2" t="s">
         <v>222</v>
       </c>
@@ -6471,14 +6490,14 @@
       </c>
       <c r="C26" s="4">
         <f>COUNTIFS('Kịch bản test'!$C$2:$C$81,"Hành trình F*",'Kịch bản test'!$K$2:$K$81,"Không đạt")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D26" s="4">
         <f>COUNTIFS('Kịch bản test'!$C$2:$C$81,"Hành trình F*",'Kịch bản test'!$K$2:$K$81,"")</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="27" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="2" t="s">
         <v>249</v>
       </c>
@@ -6492,10 +6511,10 @@
       </c>
       <c r="D27" s="4">
         <f>COUNTIFS('Kịch bản test'!$C$2:$C$81,"Hành trình G*",'Kịch bản test'!$K$2:$K$81,"")</f>
-        <v>10</v>
-      </c>
-    </row>
-    <row r="28" spans="1:4" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="2" t="s">
         <v>301</v>
       </c>
@@ -6509,10 +6528,10 @@
       </c>
       <c r="D28" s="4">
         <f>COUNTIFS('Kịch bản test'!$C$2:$C$81,"Hành trình H*",'Kịch bản test'!$K$2:$K$81,"")</f>
-        <v>5</v>
-      </c>
-    </row>
-    <row r="29" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29" spans="1:4" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2" t="s">
         <v>328</v>
       </c>
@@ -6526,10 +6545,10 @@
       </c>
       <c r="D29" s="4">
         <f>COUNTIFS('Kịch bản test'!$C$2:$C$81,"Hành trình I*",'Kịch bản test'!$K$2:$K$81,"")</f>
-        <v>8</v>
-      </c>
-    </row>
-    <row r="30" spans="1:4" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30" spans="1:4" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="2" t="s">
         <v>366</v>
       </c>
@@ -6543,10 +6562,10 @@
       </c>
       <c r="D30" s="4">
         <f>COUNTIFS('Kịch bản test'!$C$2:$C$81,"Hành trình J*",'Kịch bản test'!$K$2:$K$81,"")</f>
-        <v>7</v>
-      </c>
-    </row>
-    <row r="31" spans="1:4" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="31" spans="1:4" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2" t="s">
         <v>400</v>
       </c>
@@ -6556,11 +6575,11 @@
       </c>
       <c r="C31" s="4">
         <f>COUNTIFS('Kịch bản test'!$C$2:$C$81,"Hành trình K*",'Kịch bản test'!$K$2:$K$81,"Không đạt")</f>
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D31" s="4">
         <f>COUNTIFS('Kịch bản test'!$C$2:$C$81,"Hành trình K*",'Kịch bản test'!$K$2:$K$81,"")</f>
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -6571,152 +6590,152 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:A31"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="126" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>515</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>516</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>517</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>518</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>519</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>520</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>521</v>
       </c>
     </row>
-    <row r="9" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>522</v>
       </c>
     </row>
-    <row r="10" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>523</v>
       </c>
     </row>
-    <row r="11" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>524</v>
       </c>
     </row>
-    <row r="12" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>525</v>
       </c>
     </row>
-    <row r="13" spans="1:1" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="6" t="s">
         <v>526</v>
       </c>
     </row>
-    <row r="14" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="6" t="s">
         <v>527</v>
       </c>
     </row>
-    <row r="15" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="6" t="s">
         <v>528</v>
       </c>
     </row>
-    <row r="16" spans="1:1" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="6" t="s">
         <v>529</v>
       </c>
     </row>
-    <row r="17" spans="1:1" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>530</v>
       </c>
     </row>
-    <row r="19" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="7" t="s">
         <v>531</v>
       </c>
     </row>
-    <row r="20" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>532</v>
       </c>
     </row>
-    <row r="21" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>533</v>
       </c>
     </row>
-    <row r="22" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>534</v>
       </c>
     </row>
-    <row r="23" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>535</v>
       </c>
     </row>
-    <row r="24" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>536</v>
       </c>
     </row>
-    <row r="25" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>537</v>
       </c>
     </row>
-    <row r="26" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
         <v>538</v>
       </c>
     </row>
-    <row r="27" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
         <v>539</v>
       </c>
     </row>
-    <row r="28" spans="1:1" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
         <v>540</v>
       </c>
     </row>
-    <row r="29" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
         <v>541</v>
       </c>
     </row>
-    <row r="30" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
         <v>542</v>
       </c>
     </row>
-    <row r="31" spans="1:1" ht="70.95" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:1" ht="70.900000000000006" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="6" t="s">
         <v>543</v>
       </c>
@@ -6729,492 +6748,492 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:A101"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="126" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1" ht="24" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:1" ht="24" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="7" t="s">
         <v>544</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="7" t="s">
         <v>545</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A4" s="6" t="s">
         <v>546</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="6" t="s">
         <v>547</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A6" s="6" t="s">
         <v>548</v>
       </c>
     </row>
-    <row r="7" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="6" t="s">
         <v>549</v>
       </c>
     </row>
-    <row r="8" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="6" t="s">
         <v>550</v>
       </c>
     </row>
-    <row r="9" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A9" s="6" t="s">
         <v>551</v>
       </c>
     </row>
-    <row r="10" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
         <v>552</v>
       </c>
     </row>
-    <row r="11" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A11" s="6" t="s">
         <v>553</v>
       </c>
     </row>
-    <row r="12" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A12" s="6" t="s">
         <v>554</v>
       </c>
     </row>
-    <row r="13" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A13" s="8" t="s">
         <v>555</v>
       </c>
     </row>
-    <row r="15" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="7" t="s">
         <v>556</v>
       </c>
     </row>
-    <row r="16" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="7" t="s">
         <v>557</v>
       </c>
     </row>
-    <row r="17" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="6" t="s">
         <v>558</v>
       </c>
     </row>
-    <row r="18" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="6" t="s">
         <v>559</v>
       </c>
     </row>
-    <row r="19" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A19" s="6" t="s">
         <v>560</v>
       </c>
     </row>
-    <row r="20" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A20" s="6" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="21" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="6" t="s">
         <v>561</v>
       </c>
     </row>
-    <row r="22" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A22" s="6" t="s">
         <v>562</v>
       </c>
     </row>
-    <row r="23" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A23" s="6" t="s">
         <v>563</v>
       </c>
     </row>
-    <row r="24" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A24" s="6" t="s">
         <v>564</v>
       </c>
     </row>
-    <row r="25" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A25" s="6" t="s">
         <v>565</v>
       </c>
     </row>
-    <row r="26" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A26" s="6" t="s">
         <v>563</v>
       </c>
     </row>
-    <row r="27" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="6" t="s">
         <v>566</v>
       </c>
     </row>
-    <row r="28" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="6" t="s">
         <v>567</v>
       </c>
     </row>
-    <row r="29" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="6" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="30" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="6" t="s">
         <v>568</v>
       </c>
     </row>
-    <row r="31" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
         <v>569</v>
       </c>
     </row>
-    <row r="32" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A32" s="6" t="s">
         <v>570</v>
       </c>
     </row>
-    <row r="33" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A33" s="6" t="s">
         <v>571</v>
       </c>
     </row>
-    <row r="34" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="6" t="s">
         <v>572</v>
       </c>
     </row>
-    <row r="35" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="6" t="s">
         <v>573</v>
       </c>
     </row>
-    <row r="36" spans="1:1" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A36" s="6" t="s">
         <v>574</v>
       </c>
     </row>
-    <row r="37" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="7" t="s">
         <v>575</v>
       </c>
     </row>
-    <row r="38" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="6" t="s">
         <v>576</v>
       </c>
     </row>
-    <row r="39" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="6" t="s">
         <v>577</v>
       </c>
     </row>
-    <row r="40" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A40" s="6" t="s">
         <v>578</v>
       </c>
     </row>
-    <row r="41" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="6" t="s">
         <v>579</v>
       </c>
     </row>
-    <row r="42" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="6" t="s">
         <v>580</v>
       </c>
     </row>
-    <row r="43" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="6" t="s">
         <v>581</v>
       </c>
     </row>
-    <row r="44" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="8" t="s">
         <v>582</v>
       </c>
     </row>
-    <row r="45" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A45" s="7" t="s">
         <v>583</v>
       </c>
     </row>
-    <row r="46" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="6" t="s">
         <v>584</v>
       </c>
     </row>
-    <row r="47" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A47" s="6" t="s">
         <v>585</v>
       </c>
     </row>
-    <row r="48" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="6" t="s">
         <v>586</v>
       </c>
     </row>
-    <row r="49" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A49" s="6" t="s">
         <v>587</v>
       </c>
     </row>
-    <row r="50" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A50" s="6" t="s">
         <v>588</v>
       </c>
     </row>
-    <row r="51" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A51" s="6" t="s">
         <v>589</v>
       </c>
     </row>
-    <row r="52" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="6" t="s">
         <v>590</v>
       </c>
     </row>
-    <row r="53" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="6" t="s">
         <v>591</v>
       </c>
     </row>
-    <row r="54" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="6" t="s">
         <v>592</v>
       </c>
     </row>
-    <row r="55" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="6" t="s">
         <v>593</v>
       </c>
     </row>
-    <row r="56" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="6" t="s">
         <v>594</v>
       </c>
     </row>
-    <row r="57" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="6" t="s">
         <v>595</v>
       </c>
     </row>
-    <row r="58" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="7" t="s">
         <v>596</v>
       </c>
     </row>
-    <row r="59" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="8" t="s">
         <v>597</v>
       </c>
     </row>
-    <row r="60" spans="1:1" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="8" t="s">
         <v>598</v>
       </c>
     </row>
-    <row r="61" spans="1:1" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="6" t="s">
         <v>599</v>
       </c>
     </row>
-    <row r="62" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="6" t="s">
         <v>600</v>
       </c>
     </row>
-    <row r="63" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="6" t="s">
         <v>601</v>
       </c>
     </row>
-    <row r="64" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="6" t="s">
         <v>602</v>
       </c>
     </row>
-    <row r="65" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="6" t="s">
         <v>603</v>
       </c>
     </row>
-    <row r="66" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="6" t="s">
         <v>604</v>
       </c>
     </row>
-    <row r="67" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="6" t="s">
         <v>605</v>
       </c>
     </row>
-    <row r="68" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="6" t="s">
         <v>606</v>
       </c>
     </row>
-    <row r="69" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="6" t="s">
         <v>607</v>
       </c>
     </row>
-    <row r="70" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="6" t="s">
         <v>608</v>
       </c>
     </row>
-    <row r="71" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="6" t="s">
         <v>609</v>
       </c>
     </row>
-    <row r="72" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="6" t="s">
         <v>610</v>
       </c>
     </row>
-    <row r="73" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="6" t="s">
         <v>611</v>
       </c>
     </row>
-    <row r="74" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A74" s="6" t="s">
         <v>612</v>
       </c>
     </row>
-    <row r="75" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A75" s="6" t="s">
         <v>613</v>
       </c>
     </row>
-    <row r="76" spans="1:1" ht="44.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:1" ht="44.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A76" s="6" t="s">
         <v>614</v>
       </c>
     </row>
-    <row r="77" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A77" s="6" t="s">
         <v>615</v>
       </c>
     </row>
-    <row r="79" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A79" s="7" t="s">
         <v>616</v>
       </c>
     </row>
-    <row r="80" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A80" s="6" t="s">
         <v>617</v>
       </c>
     </row>
-    <row r="81" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A81" s="6" t="s">
         <v>618</v>
       </c>
     </row>
-    <row r="82" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A82" s="6" t="s">
         <v>619</v>
       </c>
     </row>
-    <row r="83" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A83" s="6" t="s">
         <v>620</v>
       </c>
     </row>
-    <row r="84" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A84" s="6" t="s">
         <v>621</v>
       </c>
     </row>
-    <row r="85" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A85" s="8" t="s">
         <v>622</v>
       </c>
     </row>
-    <row r="87" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A87" s="7" t="s">
         <v>623</v>
       </c>
     </row>
-    <row r="88" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A88" s="6" t="s">
         <v>624</v>
       </c>
     </row>
-    <row r="89" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A89" s="6" t="s">
         <v>625</v>
       </c>
     </row>
-    <row r="90" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A90" s="6" t="s">
         <v>626</v>
       </c>
     </row>
-    <row r="91" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A91" s="6" t="s">
         <v>627</v>
       </c>
     </row>
-    <row r="92" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A92" s="6" t="s">
         <v>628</v>
       </c>
     </row>
-    <row r="93" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A93" s="6" t="s">
         <v>629</v>
       </c>
     </row>
-    <row r="94" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A94" s="6" t="s">
         <v>630</v>
       </c>
     </row>
-    <row r="95" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A95" s="6" t="s">
         <v>631</v>
       </c>
     </row>
-    <row r="96" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A96" s="6" t="s">
         <v>632</v>
       </c>
     </row>
-    <row r="97" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A97" s="6" t="s">
         <v>633</v>
       </c>
     </row>
-    <row r="98" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A98" s="6" t="s">
         <v>634</v>
       </c>
     </row>
-    <row r="99" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A99" s="6" t="s">
         <v>635</v>
       </c>
     </row>
-    <row r="100" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:1" ht="30.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A100" s="6" t="s">
         <v>636</v>
       </c>
     </row>
-    <row r="101" spans="1:1" ht="17.399999999999999" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:1" ht="17.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A101" s="6" t="s">
         <v>637</v>
       </c>

</xml_diff>